<commit_message>
refactor: optimize project structure by moving raw images to photos/ folder and updating scripts
</commit_message>
<xml_diff>
--- a/用车费用明细.xlsx
+++ b/用车费用明细.xlsx
@@ -1787,6 +1787,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1812,6 +1815,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1837,6 +1843,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1862,6 +1871,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1887,6 +1899,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1912,6 +1927,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1937,6 +1955,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1962,6 +1983,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1987,6 +2011,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2012,6 +2039,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2037,6 +2067,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2062,6 +2095,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2087,6 +2123,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2112,6 +2151,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2137,6 +2179,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2162,6 +2207,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2187,6 +2235,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2212,6 +2263,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2237,6 +2291,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2262,6 +2319,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2281,6 +2341,534 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId63"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId64"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId65"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId66"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId67"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="68" name="Image 68" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId68"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="69" name="Image 69" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId69"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="70" name="Image 70" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId70"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="71" name="Image 71" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId71"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="72" name="Image 72" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId72"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="73" name="Image 73" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId73"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="74" name="Image 74" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId74"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="75" name="Image 75" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId75"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="76" name="Image 76" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId76"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="77" name="Image 77" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId77"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="78" name="Image 78" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId78"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="79" name="Image 79" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId79"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="80" name="Image 80" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId80"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="81" name="Image 81" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId81"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="82" name="Image 82" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId82"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="83" name="Image 83" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId83"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="84" name="Image 84" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId84"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>

</xml_diff>

<commit_message>
feat: parse toll fees from trans.pdf and fill in reimbursement xlsx
</commit_message>
<xml_diff>
--- a/用车费用明细.xlsx
+++ b/用车费用明细.xlsx
@@ -2375,6 +2375,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2400,6 +2403,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2425,6 +2431,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2450,6 +2459,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2475,6 +2487,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2500,6 +2515,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2525,6 +2543,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2550,6 +2571,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2575,6 +2599,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2600,6 +2627,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2625,6 +2655,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2650,6 +2683,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2675,6 +2711,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2700,6 +2739,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2725,6 +2767,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2750,6 +2795,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2775,6 +2823,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2800,6 +2851,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2825,6 +2879,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2850,6 +2907,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2869,6 +2929,534 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId84"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="85" name="Image 85" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId85"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="86" name="Image 86" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId86"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="87" name="Image 87" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId87"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="88" name="Image 88" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId88"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="89" name="Image 89" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId89"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="90" name="Image 90" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId90"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="91" name="Image 91" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId91"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="92" name="Image 92" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId92"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="93" name="Image 93" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId93"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="94" name="Image 94" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId94"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="95" name="Image 95" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId95"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="96" name="Image 96" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId96"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="97" name="Image 97" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId97"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="98" name="Image 98" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId98"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="99" name="Image 99" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId99"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="100" name="Image 100" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId100"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="101" name="Image 101" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId101"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="102" name="Image 102" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId102"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="103" name="Image 103" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId103"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="104" name="Image 104" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId104"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1543050" cy="2057400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="105" name="Image 105" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId105"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3324,7 +3912,9 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="n"/>
+      <c r="K5" s="4" t="n">
+        <v>86</v>
+      </c>
       <c r="L5" s="3" t="n"/>
     </row>
     <row r="6" ht="37" customHeight="1" s="42">
@@ -3358,7 +3948,9 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="n"/>
+      <c r="K6" s="4" t="n">
+        <v>76</v>
+      </c>
       <c r="L6" s="3" t="n"/>
     </row>
     <row r="7" ht="37" customHeight="1" s="42">
@@ -3392,7 +3984,9 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n"/>
-      <c r="K7" s="4" t="n"/>
+      <c r="K7" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="L7" s="3" t="n"/>
     </row>
     <row r="8" ht="37" customHeight="1" s="42">
@@ -3426,7 +4020,9 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
+      <c r="K8" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="L8" s="3" t="n"/>
     </row>
     <row r="9" ht="37" customHeight="1" s="42">
@@ -3460,7 +4056,9 @@
         <v/>
       </c>
       <c r="J9" s="4" t="n"/>
-      <c r="K9" s="4" t="n"/>
+      <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="L9" s="3" t="n"/>
     </row>
     <row r="10" ht="37" customHeight="1" s="42">
@@ -3494,7 +4092,9 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n"/>
-      <c r="K10" s="4" t="n"/>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="L10" s="3" t="n"/>
     </row>
     <row r="11" ht="37" customHeight="1" s="42">
@@ -3528,7 +4128,9 @@
         <v/>
       </c>
       <c r="J11" s="4" t="n"/>
-      <c r="K11" s="4" t="n"/>
+      <c r="K11" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="L11" s="3" t="n"/>
     </row>
     <row r="12" ht="37" customHeight="1" s="42">
@@ -3562,7 +4164,9 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="n"/>
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="L12" s="3" t="n"/>
     </row>
     <row r="13" ht="37" customHeight="1" s="42">
@@ -3596,7 +4200,9 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
+      <c r="K13" s="4" t="n">
+        <v>80.75</v>
+      </c>
       <c r="L13" s="3" t="n"/>
     </row>
     <row r="14" ht="37" customHeight="1" s="42">
@@ -3630,7 +4236,9 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
+      <c r="K14" s="4" t="n">
+        <v>73.15000000000001</v>
+      </c>
       <c r="L14" s="3" t="n"/>
     </row>
     <row r="15" ht="37" customHeight="1" s="42">
@@ -3664,7 +4272,9 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n"/>
-      <c r="K15" s="4" t="n"/>
+      <c r="K15" s="4" t="n">
+        <v>73.15000000000001</v>
+      </c>
       <c r="L15" s="3" t="n"/>
     </row>
     <row r="16" ht="37" customHeight="1" s="42">
@@ -3698,7 +4308,9 @@
         <v/>
       </c>
       <c r="J16" s="4" t="n"/>
-      <c r="K16" s="4" t="n"/>
+      <c r="K16" s="4" t="n">
+        <v>71.25</v>
+      </c>
       <c r="L16" s="3" t="n"/>
     </row>
     <row r="17" ht="37" customHeight="1" s="42">
@@ -3732,7 +4344,9 @@
         <v/>
       </c>
       <c r="J17" s="4" t="n"/>
-      <c r="K17" s="4" t="n"/>
+      <c r="K17" s="4" t="n">
+        <v>63.65</v>
+      </c>
       <c r="L17" s="3" t="n"/>
     </row>
     <row r="18" ht="39" customHeight="1" s="42">
@@ -3766,7 +4380,9 @@
         <v/>
       </c>
       <c r="J18" s="24" t="n"/>
-      <c r="K18" s="24" t="n"/>
+      <c r="K18" s="24" t="n">
+        <v>63.65</v>
+      </c>
       <c r="L18" s="25" t="n"/>
     </row>
     <row r="19" ht="29" customHeight="1" s="42">
@@ -3800,7 +4416,9 @@
         <v/>
       </c>
       <c r="J19" s="24" t="n"/>
-      <c r="K19" s="24" t="n"/>
+      <c r="K19" s="24" t="n">
+        <v>73.15000000000001</v>
+      </c>
       <c r="L19" s="25" t="n"/>
     </row>
     <row r="20" ht="34" customHeight="1" s="42">
@@ -3834,7 +4452,9 @@
         <v/>
       </c>
       <c r="J20" s="24" t="n"/>
-      <c r="K20" s="24" t="n"/>
+      <c r="K20" s="24" t="n">
+        <v>76.5</v>
+      </c>
       <c r="L20" s="25" t="n"/>
     </row>
     <row r="21" ht="32" customHeight="1" s="42">

</xml_diff>